<commit_message>
Edit drop down nama misa, fixded dropdown registrasi misa besar
</commit_message>
<xml_diff>
--- a/List Fungsionalitas Website Crembo Media.xlsx
+++ b/List Fungsionalitas Website Crembo Media.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4e51c34aafd3930f/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SURYA\UAJY\Semester 8\TA\Wireframe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{E12EA3F6-0785-4604-B8EB-DDD4ED72C8EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15929953-C4AA-44B5-A52A-67EF8A00C54C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F49FD142-BCC4-4CE2-9E02-DBAC47031907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="912" xr2:uid="{B1B77A11-58E3-4FF1-8F41-DA80BA5C2135}"/>
   </bookViews>
@@ -1295,10 +1295,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2670,7 +2666,7 @@
         <v>239</v>
       </c>
       <c r="C82" s="21" t="s">
-        <v>162</v>
+        <v>40</v>
       </c>
       <c r="D82" s="53" t="s">
         <v>265</v>

</xml_diff>